<commit_message>
feat(seeders): Script and tipos de asociaciones updated
</commit_message>
<xml_diff>
--- a/docs/Tipos_asociaciones.xlsx
+++ b/docs/Tipos_asociaciones.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvillanueva\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvillanueva\Downloads\ApiBackendCityManagement\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8533D6A-76B7-4949-9A3F-2599DFEE9C58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44068250-79C0-4DE6-A9CA-7F23BFD00088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{0A77429A-FF56-44B6-88FD-9E126A82CDCD}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId2"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$E$325</definedName>
@@ -665,7 +666,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -687,6 +688,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1047,7 +1051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>152</v>
       </c>
@@ -1064,7 +1068,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>155</v>
       </c>
@@ -1081,7 +1085,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>155</v>
       </c>
@@ -1098,7 +1102,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
         <v>152</v>
       </c>
@@ -1115,7 +1119,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
         <v>155</v>
       </c>
@@ -1132,7 +1136,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>155</v>
       </c>
@@ -1149,7 +1153,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>155</v>
       </c>
@@ -1166,7 +1170,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
         <v>152</v>
       </c>
@@ -1183,7 +1187,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
         <v>152</v>
       </c>
@@ -1200,7 +1204,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>155</v>
       </c>
@@ -1217,7 +1221,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
         <v>152</v>
       </c>
@@ -1234,7 +1238,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
         <v>152</v>
       </c>
@@ -1251,7 +1255,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>152</v>
       </c>
@@ -1268,7 +1272,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>152</v>
       </c>
@@ -1285,7 +1289,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>152</v>
       </c>
@@ -1302,7 +1306,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>152</v>
       </c>
@@ -1319,7 +1323,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>152</v>
       </c>
@@ -1336,7 +1340,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>152</v>
       </c>
@@ -1353,7 +1357,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>152</v>
       </c>
@@ -1370,7 +1374,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>152</v>
       </c>
@@ -1387,7 +1391,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>152</v>
       </c>
@@ -1404,7 +1408,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>152</v>
       </c>
@@ -1421,7 +1425,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" ht="25" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>155</v>
       </c>
@@ -1434,11 +1438,11 @@
       <c r="D24" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>155</v>
       </c>
@@ -1455,7 +1459,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>152</v>
       </c>
@@ -1472,7 +1476,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>155</v>
       </c>
@@ -1489,7 +1493,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
         <v>152</v>
       </c>
@@ -1506,7 +1510,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>152</v>
       </c>
@@ -1523,7 +1527,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
         <v>155</v>
       </c>
@@ -1540,7 +1544,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
         <v>152</v>
       </c>
@@ -1557,7 +1561,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
         <v>152</v>
       </c>
@@ -1574,7 +1578,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>155</v>
       </c>
@@ -1591,7 +1595,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="34" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
         <v>155</v>
       </c>
@@ -1608,7 +1612,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="35" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
         <v>155</v>
       </c>
@@ -1625,7 +1629,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="36" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
         <v>155</v>
       </c>
@@ -1642,7 +1646,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="37" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
         <v>155</v>
       </c>
@@ -1659,7 +1663,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="38" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
         <v>155</v>
       </c>
@@ -1676,7 +1680,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="39" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
         <v>155</v>
       </c>
@@ -1693,7 +1697,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="40" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="3" t="s">
         <v>155</v>
       </c>
@@ -1710,7 +1714,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="41" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
         <v>155</v>
       </c>
@@ -1727,7 +1731,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="42" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
         <v>155</v>
       </c>
@@ -1744,7 +1748,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="43" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
         <v>155</v>
       </c>
@@ -1761,7 +1765,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="44" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
         <v>155</v>
       </c>
@@ -1778,7 +1782,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="45" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
         <v>155</v>
       </c>
@@ -1795,7 +1799,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="46" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
         <v>155</v>
       </c>
@@ -1812,7 +1816,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="47" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
         <v>155</v>
       </c>
@@ -1829,7 +1833,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="48" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
         <v>155</v>
       </c>
@@ -1846,7 +1850,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
         <v>152</v>
       </c>
@@ -1861,7 +1865,7 @@
       </c>
       <c r="E49" s="6"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
         <v>152</v>
       </c>
@@ -1878,7 +1882,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>155</v>
       </c>
@@ -1895,7 +1899,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
         <v>152</v>
       </c>
@@ -1912,7 +1916,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
         <v>154</v>
       </c>
@@ -1929,7 +1933,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
         <v>154</v>
       </c>
@@ -1946,7 +1950,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
         <v>152</v>
       </c>
@@ -1963,7 +1967,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
         <v>152</v>
       </c>
@@ -1980,7 +1984,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
         <v>152</v>
       </c>
@@ -1997,7 +2001,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
         <v>152</v>
       </c>
@@ -2014,7 +2018,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
         <v>152</v>
       </c>
@@ -2031,7 +2035,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
         <v>152</v>
       </c>
@@ -2048,7 +2052,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
         <v>152</v>
       </c>
@@ -2065,7 +2069,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
         <v>152</v>
       </c>
@@ -2082,7 +2086,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
         <v>154</v>
       </c>
@@ -2099,7 +2103,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
         <v>154</v>
       </c>
@@ -2116,7 +2120,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
         <v>154</v>
       </c>
@@ -2133,7 +2137,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
         <v>154</v>
       </c>
@@ -2150,7 +2154,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
         <v>154</v>
       </c>
@@ -2167,7 +2171,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
         <v>154</v>
       </c>
@@ -2184,7 +2188,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
         <v>154</v>
       </c>
@@ -2201,7 +2205,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="3" t="s">
         <v>152</v>
       </c>
@@ -2218,7 +2222,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="3" t="s">
         <v>152</v>
       </c>
@@ -2235,7 +2239,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="3" t="s">
         <v>152</v>
       </c>
@@ -2252,7 +2256,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="3" t="s">
         <v>152</v>
       </c>
@@ -2269,7 +2273,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="3" t="s">
         <v>152</v>
       </c>
@@ -2286,7 +2290,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="3" t="s">
         <v>152</v>
       </c>
@@ -2303,7 +2307,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="3" t="s">
         <v>152</v>
       </c>
@@ -2320,7 +2324,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="3" t="s">
         <v>152</v>
       </c>
@@ -2337,7 +2341,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="3" t="s">
         <v>152</v>
       </c>
@@ -2354,7 +2358,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="3" t="s">
         <v>152</v>
       </c>
@@ -2371,7 +2375,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="3" t="s">
         <v>152</v>
       </c>
@@ -2388,7 +2392,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="3" t="s">
         <v>152</v>
       </c>
@@ -2405,7 +2409,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="3" t="s">
         <v>152</v>
       </c>
@@ -2422,7 +2426,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="3" t="s">
         <v>152</v>
       </c>
@@ -2439,7 +2443,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="3" t="s">
         <v>152</v>
       </c>
@@ -2456,7 +2460,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="3" t="s">
         <v>152</v>
       </c>
@@ -2473,7 +2477,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="3" t="s">
         <v>152</v>
       </c>
@@ -2490,7 +2494,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="3" t="s">
         <v>152</v>
       </c>
@@ -2507,7 +2511,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
         <v>152</v>
       </c>
@@ -2524,7 +2528,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="3" t="s">
         <v>152</v>
       </c>
@@ -2541,7 +2545,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="3" t="s">
         <v>152</v>
       </c>
@@ -2558,7 +2562,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="3" t="s">
         <v>152</v>
       </c>
@@ -2575,7 +2579,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="3" t="s">
         <v>152</v>
       </c>
@@ -2592,7 +2596,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="3" t="s">
         <v>152</v>
       </c>
@@ -2609,7 +2613,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="3" t="s">
         <v>152</v>
       </c>
@@ -2626,7 +2630,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="3" t="s">
         <v>152</v>
       </c>
@@ -2643,7 +2647,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="3" t="s">
         <v>152</v>
       </c>
@@ -2660,7 +2664,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="3" t="s">
         <v>152</v>
       </c>
@@ -2677,7 +2681,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="3" t="s">
         <v>152</v>
       </c>
@@ -2694,7 +2698,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="3" t="s">
         <v>152</v>
       </c>
@@ -2711,7 +2715,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="3" t="s">
         <v>154</v>
       </c>
@@ -2728,7 +2732,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="101" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="3" t="s">
         <v>155</v>
       </c>
@@ -2745,7 +2749,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="3" t="s">
         <v>152</v>
       </c>
@@ -2762,7 +2766,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="3" t="s">
         <v>154</v>
       </c>
@@ -2779,7 +2783,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="3" t="s">
         <v>152</v>
       </c>
@@ -2796,7 +2800,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="3" t="s">
         <v>152</v>
       </c>
@@ -2813,7 +2817,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="106" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="3" t="s">
         <v>155</v>
       </c>
@@ -2830,7 +2834,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="3" t="s">
         <v>152</v>
       </c>
@@ -2847,7 +2851,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="3" t="s">
         <v>152</v>
       </c>
@@ -2864,7 +2868,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="3" t="s">
         <v>152</v>
       </c>
@@ -2881,7 +2885,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="3" t="s">
         <v>152</v>
       </c>
@@ -2898,7 +2902,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="3" t="s">
         <v>152</v>
       </c>
@@ -2915,7 +2919,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="3" t="s">
         <v>152</v>
       </c>
@@ -2932,7 +2936,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="3" t="s">
         <v>152</v>
       </c>
@@ -2949,7 +2953,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="3" t="s">
         <v>152</v>
       </c>
@@ -2966,7 +2970,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="3" t="s">
         <v>152</v>
       </c>
@@ -2983,7 +2987,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="3" t="s">
         <v>152</v>
       </c>
@@ -3000,7 +3004,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="3" t="s">
         <v>152</v>
       </c>
@@ -3017,7 +3021,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="3" t="s">
         <v>152</v>
       </c>
@@ -3034,7 +3038,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="3" t="s">
         <v>152</v>
       </c>
@@ -3051,7 +3055,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="3" t="s">
         <v>152</v>
       </c>
@@ -3068,7 +3072,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="3" t="s">
         <v>152</v>
       </c>
@@ -3085,7 +3089,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="3" t="s">
         <v>152</v>
       </c>
@@ -3102,7 +3106,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="3" t="s">
         <v>152</v>
       </c>
@@ -3119,7 +3123,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="3" t="s">
         <v>152</v>
       </c>
@@ -3136,7 +3140,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="3" t="s">
         <v>152</v>
       </c>
@@ -3153,7 +3157,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="3" t="s">
         <v>152</v>
       </c>
@@ -3170,7 +3174,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="3" t="s">
         <v>152</v>
       </c>
@@ -3187,7 +3191,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="3" t="s">
         <v>152</v>
       </c>
@@ -3204,7 +3208,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="3" t="s">
         <v>152</v>
       </c>
@@ -3221,7 +3225,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="3" t="s">
         <v>152</v>
       </c>
@@ -3238,7 +3242,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="3" t="s">
         <v>152</v>
       </c>
@@ -3255,7 +3259,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="3" t="s">
         <v>152</v>
       </c>
@@ -3272,7 +3276,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="3" t="s">
         <v>152</v>
       </c>
@@ -3289,7 +3293,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="3" t="s">
         <v>152</v>
       </c>
@@ -3306,7 +3310,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="3" t="s">
         <v>152</v>
       </c>
@@ -3323,7 +3327,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="3" t="s">
         <v>152</v>
       </c>
@@ -3340,7 +3344,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="3" t="s">
         <v>152</v>
       </c>
@@ -3357,7 +3361,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="3" t="s">
         <v>152</v>
       </c>
@@ -3374,7 +3378,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="3" t="s">
         <v>154</v>
       </c>
@@ -3391,7 +3395,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="3" t="s">
         <v>152</v>
       </c>
@@ -3408,7 +3412,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="3" t="s">
         <v>154</v>
       </c>
@@ -3425,7 +3429,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" s="3" t="s">
         <v>154</v>
       </c>
@@ -3442,7 +3446,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="3" t="s">
         <v>152</v>
       </c>
@@ -3459,7 +3463,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="3" t="s">
         <v>154</v>
       </c>
@@ -3476,7 +3480,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="3" t="s">
         <v>154</v>
       </c>
@@ -3493,7 +3497,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="3" t="s">
         <v>154</v>
       </c>
@@ -3510,7 +3514,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="3" t="s">
         <v>154</v>
       </c>
@@ -3527,7 +3531,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="3" t="s">
         <v>154</v>
       </c>
@@ -3544,7 +3548,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="3" t="s">
         <v>154</v>
       </c>
@@ -3561,7 +3565,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="3" t="s">
         <v>154</v>
       </c>
@@ -3578,7 +3582,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="151" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="3" t="s">
         <v>155</v>
       </c>
@@ -3595,7 +3599,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="152" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="3" t="s">
         <v>155</v>
       </c>
@@ -3612,7 +3616,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" s="3" t="s">
         <v>154</v>
       </c>
@@ -3629,7 +3633,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" s="3" t="s">
         <v>152</v>
       </c>
@@ -3646,7 +3650,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" s="3" t="s">
         <v>152</v>
       </c>
@@ -3663,7 +3667,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" s="3" t="s">
         <v>154</v>
       </c>
@@ -3680,7 +3684,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" s="3" t="s">
         <v>154</v>
       </c>
@@ -3697,7 +3701,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="3" t="s">
         <v>154</v>
       </c>
@@ -3714,7 +3718,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="3" t="s">
         <v>154</v>
       </c>
@@ -3731,7 +3735,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="160" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="3" t="s">
         <v>155</v>
       </c>
@@ -3748,7 +3752,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="161" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="3" t="s">
         <v>155</v>
       </c>
@@ -3765,7 +3769,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="162" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="3" t="s">
         <v>155</v>
       </c>
@@ -3782,7 +3786,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="163" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="3" t="s">
         <v>155</v>
       </c>
@@ -3799,7 +3803,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="164" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="3" t="s">
         <v>155</v>
       </c>
@@ -3816,7 +3820,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" s="3" t="s">
         <v>152</v>
       </c>
@@ -3833,7 +3837,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" s="3" t="s">
         <v>152</v>
       </c>
@@ -3850,7 +3854,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" s="3" t="s">
         <v>152</v>
       </c>
@@ -3867,7 +3871,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" s="3" t="s">
         <v>152</v>
       </c>
@@ -3884,7 +3888,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" s="3" t="s">
         <v>152</v>
       </c>
@@ -3901,7 +3905,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" s="3" t="s">
         <v>152</v>
       </c>
@@ -3918,7 +3922,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" s="3" t="s">
         <v>152</v>
       </c>
@@ -3935,7 +3939,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" s="3" t="s">
         <v>152</v>
       </c>
@@ -3952,7 +3956,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" s="3" t="s">
         <v>152</v>
       </c>
@@ -3969,7 +3973,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" s="3" t="s">
         <v>152</v>
       </c>
@@ -3986,7 +3990,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" s="3" t="s">
         <v>152</v>
       </c>
@@ -4003,7 +4007,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" s="3" t="s">
         <v>152</v>
       </c>
@@ -4020,7 +4024,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="3" t="s">
         <v>152</v>
       </c>
@@ -4037,7 +4041,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" s="3" t="s">
         <v>152</v>
       </c>
@@ -4054,7 +4058,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" s="3" t="s">
         <v>152</v>
       </c>
@@ -4071,7 +4075,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" s="3" t="s">
         <v>152</v>
       </c>
@@ -4088,7 +4092,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="3" t="s">
         <v>152</v>
       </c>
@@ -4105,7 +4109,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="182" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="3" t="s">
         <v>155</v>
       </c>
@@ -4122,7 +4126,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="3" t="s">
         <v>152</v>
       </c>
@@ -4139,7 +4143,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" s="3" t="s">
         <v>152</v>
       </c>
@@ -4156,7 +4160,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" s="3" t="s">
         <v>152</v>
       </c>
@@ -4173,7 +4177,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" s="3" t="s">
         <v>152</v>
       </c>
@@ -4190,7 +4194,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" s="3" t="s">
         <v>152</v>
       </c>
@@ -4207,7 +4211,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" s="3" t="s">
         <v>152</v>
       </c>
@@ -4224,7 +4228,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" s="3" t="s">
         <v>152</v>
       </c>
@@ -4241,7 +4245,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" s="3" t="s">
         <v>152</v>
       </c>
@@ -4258,7 +4262,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" s="3" t="s">
         <v>152</v>
       </c>
@@ -4275,7 +4279,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" s="3" t="s">
         <v>152</v>
       </c>
@@ -4292,7 +4296,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" s="3" t="s">
         <v>152</v>
       </c>
@@ -4309,7 +4313,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" s="3" t="s">
         <v>152</v>
       </c>
@@ -4326,7 +4330,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" s="3" t="s">
         <v>152</v>
       </c>
@@ -4343,7 +4347,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" s="3" t="s">
         <v>152</v>
       </c>
@@ -4360,7 +4364,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" s="3" t="s">
         <v>152</v>
       </c>
@@ -4377,7 +4381,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" s="3" t="s">
         <v>152</v>
       </c>
@@ -4394,7 +4398,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" s="3" t="s">
         <v>152</v>
       </c>
@@ -4411,7 +4415,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" s="3" t="s">
         <v>152</v>
       </c>
@@ -4428,7 +4432,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" s="3" t="s">
         <v>152</v>
       </c>
@@ -4445,7 +4449,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" s="3" t="s">
         <v>152</v>
       </c>
@@ -4462,7 +4466,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" s="3" t="s">
         <v>152</v>
       </c>
@@ -4479,7 +4483,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" s="3" t="s">
         <v>152</v>
       </c>
@@ -4496,7 +4500,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" s="3" t="s">
         <v>152</v>
       </c>
@@ -4513,7 +4517,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" s="3" t="s">
         <v>152</v>
       </c>
@@ -4530,7 +4534,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" s="3" t="s">
         <v>152</v>
       </c>
@@ -4547,7 +4551,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" s="3" t="s">
         <v>152</v>
       </c>
@@ -4564,7 +4568,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" s="3" t="s">
         <v>152</v>
       </c>
@@ -4581,7 +4585,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" s="3" t="s">
         <v>152</v>
       </c>
@@ -4598,7 +4602,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" s="3" t="s">
         <v>152</v>
       </c>
@@ -4615,7 +4619,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" s="3" t="s">
         <v>152</v>
       </c>
@@ -4632,7 +4636,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" s="3" t="s">
         <v>152</v>
       </c>
@@ -4649,7 +4653,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" s="3" t="s">
         <v>152</v>
       </c>
@@ -4666,7 +4670,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" s="3" t="s">
         <v>152</v>
       </c>
@@ -4683,7 +4687,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" s="3" t="s">
         <v>152</v>
       </c>
@@ -4700,7 +4704,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" s="3" t="s">
         <v>152</v>
       </c>
@@ -4717,7 +4721,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" s="3" t="s">
         <v>152</v>
       </c>
@@ -4734,7 +4738,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" s="3" t="s">
         <v>152</v>
       </c>
@@ -4751,7 +4755,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" s="3" t="s">
         <v>152</v>
       </c>
@@ -4768,7 +4772,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" s="3" t="s">
         <v>152</v>
       </c>
@@ -4785,7 +4789,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" s="3" t="s">
         <v>152</v>
       </c>
@@ -4802,7 +4806,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" s="3" t="s">
         <v>152</v>
       </c>
@@ -4819,7 +4823,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" s="3" t="s">
         <v>152</v>
       </c>
@@ -4836,7 +4840,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" s="3" t="s">
         <v>152</v>
       </c>
@@ -4853,7 +4857,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" s="3" t="s">
         <v>152</v>
       </c>
@@ -4870,7 +4874,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" s="3" t="s">
         <v>152</v>
       </c>
@@ -4887,7 +4891,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" s="3" t="s">
         <v>152</v>
       </c>
@@ -4904,7 +4908,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" s="3" t="s">
         <v>152</v>
       </c>
@@ -4921,7 +4925,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" s="3" t="s">
         <v>152</v>
       </c>
@@ -4938,7 +4942,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" s="3" t="s">
         <v>152</v>
       </c>
@@ -4955,7 +4959,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="232" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A232" s="3" t="s">
         <v>155</v>
       </c>
@@ -4972,7 +4976,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="233" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A233" s="3" t="s">
         <v>155</v>
       </c>
@@ -4989,7 +4993,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="234" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A234" s="3" t="s">
         <v>155</v>
       </c>
@@ -5006,7 +5010,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="235" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A235" s="3" t="s">
         <v>155</v>
       </c>
@@ -5023,7 +5027,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="236" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A236" s="3" t="s">
         <v>155</v>
       </c>
@@ -5040,7 +5044,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="237" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A237" s="3" t="s">
         <v>155</v>
       </c>
@@ -5057,7 +5061,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="238" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A238" s="3" t="s">
         <v>155</v>
       </c>
@@ -5074,7 +5078,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="239" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A239" s="3" t="s">
         <v>155</v>
       </c>
@@ -5091,7 +5095,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="240" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A240" s="3" t="s">
         <v>155</v>
       </c>
@@ -5108,7 +5112,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="241" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A241" s="3" t="s">
         <v>155</v>
       </c>
@@ -5125,7 +5129,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="242" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A242" s="3" t="s">
         <v>155</v>
       </c>
@@ -5142,7 +5146,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="243" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A243" s="3" t="s">
         <v>155</v>
       </c>
@@ -5159,7 +5163,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="244" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A244" s="3" t="s">
         <v>155</v>
       </c>
@@ -5176,7 +5180,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="245" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A245" s="3" t="s">
         <v>155</v>
       </c>
@@ -5193,7 +5197,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="246" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A246" s="3" t="s">
         <v>155</v>
       </c>
@@ -5210,7 +5214,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="247" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A247" s="3" t="s">
         <v>155</v>
       </c>
@@ -5227,7 +5231,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" s="3" t="s">
         <v>152</v>
       </c>
@@ -5244,7 +5248,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="249" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A249" s="3" t="s">
         <v>155</v>
       </c>
@@ -5261,7 +5265,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="250" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A250" s="3" t="s">
         <v>155</v>
       </c>
@@ -5278,7 +5282,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="251" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A251" s="3" t="s">
         <v>155</v>
       </c>
@@ -5295,7 +5299,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="252" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A252" s="3" t="s">
         <v>155</v>
       </c>
@@ -5312,7 +5316,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="253" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A253" s="3" t="s">
         <v>155</v>
       </c>
@@ -5329,7 +5333,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="254" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A254" s="3" t="s">
         <v>155</v>
       </c>
@@ -5346,7 +5350,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="255" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A255" s="3" t="s">
         <v>155</v>
       </c>
@@ -5363,7 +5367,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="256" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A256" s="3" t="s">
         <v>155</v>
       </c>
@@ -5380,7 +5384,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="257" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A257" s="3" t="s">
         <v>155</v>
       </c>
@@ -5397,7 +5401,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="258" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A258" s="3" t="s">
         <v>155</v>
       </c>
@@ -5414,7 +5418,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="259" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A259" s="3" t="s">
         <v>155</v>
       </c>
@@ -5431,7 +5435,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="260" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A260" s="3" t="s">
         <v>155</v>
       </c>
@@ -5448,7 +5452,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="261" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A261" s="3" t="s">
         <v>155</v>
       </c>
@@ -5465,7 +5469,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="262" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A262" s="3" t="s">
         <v>155</v>
       </c>
@@ -5482,7 +5486,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="263" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A263" s="3" t="s">
         <v>155</v>
       </c>
@@ -5499,7 +5503,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="264" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A264" s="3" t="s">
         <v>155</v>
       </c>
@@ -5516,7 +5520,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="265" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A265" s="3" t="s">
         <v>155</v>
       </c>
@@ -5533,7 +5537,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="266" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A266" s="3" t="s">
         <v>155</v>
       </c>
@@ -5550,7 +5554,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="267" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A267" s="3" t="s">
         <v>155</v>
       </c>
@@ -5567,7 +5571,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="268" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A268" s="3" t="s">
         <v>155</v>
       </c>
@@ -5584,7 +5588,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="269" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A269" s="3" t="s">
         <v>155</v>
       </c>
@@ -5601,7 +5605,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="270" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A270" s="3" t="s">
         <v>155</v>
       </c>
@@ -5618,7 +5622,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="271" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A271" s="3" t="s">
         <v>155</v>
       </c>
@@ -5635,7 +5639,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="272" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A272" s="3" t="s">
         <v>155</v>
       </c>
@@ -5652,7 +5656,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="273" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A273" s="3" t="s">
         <v>155</v>
       </c>
@@ -5669,7 +5673,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="274" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A274" s="3" t="s">
         <v>155</v>
       </c>
@@ -5686,7 +5690,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="275" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A275" s="3" t="s">
         <v>155</v>
       </c>
@@ -5703,7 +5707,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="276" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A276" s="3" t="s">
         <v>155</v>
       </c>
@@ -5720,7 +5724,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="277" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A277" s="3" t="s">
         <v>155</v>
       </c>
@@ -5737,7 +5741,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="278" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A278" s="3" t="s">
         <v>155</v>
       </c>
@@ -5754,7 +5758,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="279" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A279" s="3" t="s">
         <v>155</v>
       </c>
@@ -5771,7 +5775,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="280" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A280" s="3" t="s">
         <v>155</v>
       </c>
@@ -5788,7 +5792,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="281" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A281" s="3" t="s">
         <v>155</v>
       </c>
@@ -5805,7 +5809,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="282" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A282" s="3" t="s">
         <v>155</v>
       </c>
@@ -5822,7 +5826,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="283" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A283" s="3" t="s">
         <v>155</v>
       </c>
@@ -5839,7 +5843,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="284" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A284" s="3" t="s">
         <v>155</v>
       </c>
@@ -5856,7 +5860,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="285" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A285" s="3" t="s">
         <v>155</v>
       </c>
@@ -5873,7 +5877,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="286" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A286" s="3" t="s">
         <v>155</v>
       </c>
@@ -5890,7 +5894,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="287" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A287" s="3" t="s">
         <v>155</v>
       </c>
@@ -5907,7 +5911,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="288" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A288" s="3" t="s">
         <v>155</v>
       </c>
@@ -5924,7 +5928,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="289" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A289" s="3" t="s">
         <v>155</v>
       </c>
@@ -5941,7 +5945,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="290" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A290" s="3" t="s">
         <v>155</v>
       </c>
@@ -5958,7 +5962,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="291" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A291" s="3" t="s">
         <v>155</v>
       </c>
@@ -5975,7 +5979,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="292" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A292" s="3" t="s">
         <v>155</v>
       </c>
@@ -5992,7 +5996,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="293" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A293" s="3" t="s">
         <v>155</v>
       </c>
@@ -6009,7 +6013,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="294" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A294" s="3" t="s">
         <v>155</v>
       </c>
@@ -6026,7 +6030,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="295" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A295" s="3" t="s">
         <v>155</v>
       </c>
@@ -6043,7 +6047,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="296" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A296" s="3" t="s">
         <v>155</v>
       </c>
@@ -6060,7 +6064,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="297" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A297" s="3" t="s">
         <v>155</v>
       </c>
@@ -6077,7 +6081,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="298" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A298" s="3" t="s">
         <v>155</v>
       </c>
@@ -6094,7 +6098,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="299" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A299" s="3" t="s">
         <v>155</v>
       </c>
@@ -6111,7 +6115,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="300" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A300" s="3" t="s">
         <v>155</v>
       </c>
@@ -6128,7 +6132,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="301" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A301" s="3" t="s">
         <v>155</v>
       </c>
@@ -6145,7 +6149,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="302" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A302" s="3" t="s">
         <v>155</v>
       </c>
@@ -6162,7 +6166,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="303" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A303" s="3" t="s">
         <v>155</v>
       </c>
@@ -6179,7 +6183,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="304" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A304" s="3" t="s">
         <v>155</v>
       </c>
@@ -6196,7 +6200,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="305" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A305" s="3" t="s">
         <v>155</v>
       </c>
@@ -6213,7 +6217,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="306" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A306" s="3" t="s">
         <v>155</v>
       </c>
@@ -6230,7 +6234,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="307" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A307" s="3" t="s">
         <v>155</v>
       </c>
@@ -6247,7 +6251,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="308" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A308" s="3" t="s">
         <v>155</v>
       </c>
@@ -6264,7 +6268,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="309" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A309" s="3" t="s">
         <v>155</v>
       </c>
@@ -6281,7 +6285,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="310" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A310" s="3" t="s">
         <v>155</v>
       </c>
@@ -6298,7 +6302,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="311" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A311" s="3" t="s">
         <v>155</v>
       </c>
@@ -6315,7 +6319,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="312" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A312" s="3" t="s">
         <v>155</v>
       </c>
@@ -6332,7 +6336,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="313" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A313" s="3" t="s">
         <v>155</v>
       </c>
@@ -6349,7 +6353,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="314" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A314" s="3" t="s">
         <v>155</v>
       </c>
@@ -6366,7 +6370,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="315" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A315" s="3" t="s">
         <v>155</v>
       </c>
@@ -6383,7 +6387,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="316" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A316" s="3" t="s">
         <v>155</v>
       </c>
@@ -6400,7 +6404,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="317" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A317" s="3" t="s">
         <v>155</v>
       </c>
@@ -6417,7 +6421,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="318" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A318" s="3" t="s">
         <v>155</v>
       </c>
@@ -6434,7 +6438,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="319" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A319" s="3" t="s">
         <v>155</v>
       </c>
@@ -6451,7 +6455,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="320" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A320" s="3" t="s">
         <v>155</v>
       </c>
@@ -6468,7 +6472,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="321" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A321" s="3" t="s">
         <v>155</v>
       </c>
@@ -6485,7 +6489,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
       <c r="A322" s="3" t="s">
         <v>152</v>
       </c>
@@ -6502,7 +6506,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="323" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A323" s="3" t="s">
         <v>155</v>
       </c>
@@ -6519,7 +6523,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="324" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A324" s="3" t="s">
         <v>155</v>
       </c>
@@ -6536,7 +6540,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="325" spans="1:5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A325" s="3" t="s">
         <v>155</v>
       </c>
@@ -6557,8 +6561,7 @@
   <autoFilter ref="A1:E325" xr:uid="{2566881A-A4AF-4342-850D-3A2B124C31B1}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Consorcio"/>
-        <filter val="Union temporal"/>
+        <filter val="Juridica"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -6567,6 +6570,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{813850AE-4079-4994-AC31-997168BC2F49}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2427147E-9754-4F57-8F8E-27DC2118D8DC}">
   <dimension ref="B1:C196"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>